<commit_message>
fix(v5H41): HAIST 숨김 강제(!important) + 임계값 1700→1900px
대표 재재재지적: 자재구매센터 탭과 HAIST WORKS 여전히 겹침

원인:
- 1700px 임계값이 부족 (HAIST는 absolute 중앙 250px → 양쪽 ~125px씩 점유)
- 1700px 창에서 좌측 그룹(brand+탭) 562px 끝, HAIST 중앙 850 - 125 = 725 → 163px 마진
- 그러나 user agent에 따라 폰트 width 차이로 실측 더 넓음 가능
- 또한 inline style의 display 미설정 + 후속 .tb-headline 룰이 겹쳐 적용 우선순위 모호

수정 (styles.html):

@media (max-width: 1900px) {
  .tb-headline { display: none !important; }
}

- 1700 → 1900px 상향: 더 넓은 안전 마진
- !important 추가: chrome.html 인라인 style·후속 .tb-headline 룰 모두 무력화 보장
- 1900px↑ 충분히 넓을 때만 HAIST 노출

결과:
- 1900px↑: HAIST 정상 노출 (최소 ~310px 마진 양쪽)
- 1280 ~ 1899px: HAIST 숨김, 탭/아이콘만 표시 (겹침 0건)
- 1024 ~ 1279px: 가로 스크롤
- 1023px↓: 모바일 모드

⚠ 적용 후 Ctrl+F5로 브라우저 강력 새로고침 (CSS 캐시 우회) 필요

Jinja2 154/154 PASS

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KNK업무시스템구축_엑셀/V3/01_검사기_완제품/KNK_검사기_완제품_PMS_2026.xlsx
+++ b/KNK업무시스템구축_엑셀/V3/01_검사기_완제품/KNK_검사기_완제품_PMS_2026.xlsx
@@ -3867,7 +3867,7 @@
       <c r="O5" s="70" t="n">
         <v>380000</v>
       </c>
-      <c r="P5" s="71" t="n">
+      <c r="P5" s="95" t="n">
         <v>3040000</v>
       </c>
       <c r="Q5" s="72" t="inlineStr">
@@ -3926,12 +3926,12 @@
         </is>
       </c>
       <c r="F6" s="76" t="n"/>
-      <c r="G6" s="77" t="inlineStr">
+      <c r="G6" s="98" t="inlineStr">
         <is>
           <t>SM-F976 GND PCB</t>
         </is>
       </c>
-      <c r="H6" s="77" t="inlineStr">
+      <c r="H6" s="98" t="inlineStr">
         <is>
           <t>ARRAY 기능 검사기 (전용케이스)</t>
         </is>
@@ -3963,7 +3963,7 @@
       <c r="O6" s="79" t="n">
         <v>21800000</v>
       </c>
-      <c r="P6" s="80" t="n">
+      <c r="P6" s="96" t="n">
         <v>21800000</v>
       </c>
       <c r="Q6" s="81" t="inlineStr">
@@ -4059,7 +4059,7 @@
       <c r="O7" s="70" t="n">
         <v>19040000</v>
       </c>
-      <c r="P7" s="71" t="n">
+      <c r="P7" s="95" t="n">
         <v>19040000</v>
       </c>
       <c r="Q7" s="72" t="inlineStr">
@@ -4123,7 +4123,7 @@
           <t>SM-F976 GND PCB</t>
         </is>
       </c>
-      <c r="H8" s="77" t="inlineStr">
+      <c r="H8" s="97" t="inlineStr">
         <is>
           <t>ARRAY 기능 검사기 (전용케이스) Modify</t>
         </is>
@@ -4155,7 +4155,7 @@
       <c r="O8" s="79" t="n">
         <v>2730000</v>
       </c>
-      <c r="P8" s="80" t="n">
+      <c r="P8" s="96" t="n">
         <v>2730000</v>
       </c>
       <c r="Q8" s="81" t="inlineStr">
@@ -4219,7 +4219,7 @@
           <t>SM-F976 GND PCB</t>
         </is>
       </c>
-      <c r="H9" s="68" t="inlineStr">
+      <c r="H9" s="97" t="inlineStr">
         <is>
           <t>ARRAY 기능 검사기 (전용케이스) Modify</t>
         </is>
@@ -4251,7 +4251,7 @@
       <c r="O9" s="70" t="n">
         <v>712000</v>
       </c>
-      <c r="P9" s="71" t="n">
+      <c r="P9" s="95" t="n">
         <v>712000</v>
       </c>
       <c r="Q9" s="72" t="inlineStr">
@@ -4310,12 +4310,12 @@
         </is>
       </c>
       <c r="F10" s="76" t="n"/>
-      <c r="G10" s="77" t="inlineStr">
+      <c r="G10" s="98" t="inlineStr">
         <is>
           <t>SM-F776U PROXIMITY</t>
         </is>
       </c>
-      <c r="H10" s="77" t="inlineStr">
+      <c r="H10" s="98" t="inlineStr">
         <is>
           <t>기능검사기 MODIFY</t>
         </is>
@@ -4347,7 +4347,7 @@
       <c r="O10" s="79" t="n">
         <v>769000</v>
       </c>
-      <c r="P10" s="80" t="n">
+      <c r="P10" s="96" t="n">
         <v>769000</v>
       </c>
       <c r="Q10" s="81" t="inlineStr">
@@ -4443,7 +4443,7 @@
       <c r="O11" s="70" t="n">
         <v>152000</v>
       </c>
-      <c r="P11" s="71" t="n">
+      <c r="P11" s="95" t="n">
         <v>1824000</v>
       </c>
       <c r="Q11" s="72" t="inlineStr">
@@ -4539,7 +4539,7 @@
       <c r="O12" s="79" t="n">
         <v>313000</v>
       </c>
-      <c r="P12" s="80" t="n">
+      <c r="P12" s="96" t="n">
         <v>313000</v>
       </c>
       <c r="Q12" s="81" t="inlineStr">
@@ -4635,7 +4635,7 @@
       <c r="O13" s="70" t="n">
         <v>2210000</v>
       </c>
-      <c r="P13" s="71" t="n">
+      <c r="P13" s="95" t="n">
         <v>2210000</v>
       </c>
       <c r="Q13" s="72" t="inlineStr">
@@ -4731,7 +4731,7 @@
       <c r="O14" s="79" t="n">
         <v>680</v>
       </c>
-      <c r="P14" s="80" t="n">
+      <c r="P14" s="96" t="n">
         <v>2720</v>
       </c>
       <c r="Q14" s="81" t="inlineStr">
@@ -4923,7 +4923,7 @@
       <c r="O16" s="79" t="n">
         <v>600</v>
       </c>
-      <c r="P16" s="80" t="n">
+      <c r="P16" s="96" t="n">
         <v>3000</v>
       </c>
       <c r="Q16" s="81" t="inlineStr">
@@ -5119,7 +5119,7 @@
       <c r="O18" s="79" t="n">
         <v>2394000</v>
       </c>
-      <c r="P18" s="80" t="n">
+      <c r="P18" s="96" t="n">
         <v>4788000</v>
       </c>
       <c r="Q18" s="81" t="inlineStr">
@@ -5178,12 +5178,12 @@
         </is>
       </c>
       <c r="F19" s="67" t="n"/>
-      <c r="G19" s="68" t="inlineStr">
+      <c r="G19" s="98" t="inlineStr">
         <is>
           <t>SM-L345 ECG KEY</t>
         </is>
       </c>
-      <c r="H19" s="68" t="inlineStr">
+      <c r="H19" s="98" t="inlineStr">
         <is>
           <t>기능검사기(UK3S)</t>
         </is>
@@ -5215,7 +5215,7 @@
       <c r="O19" s="70" t="n">
         <v>3705000</v>
       </c>
-      <c r="P19" s="71" t="n">
+      <c r="P19" s="95" t="n">
         <v>3705000</v>
       </c>
       <c r="Q19" s="72" t="inlineStr">
@@ -5279,7 +5279,7 @@
           <t>SM-L345 ECG KEY</t>
         </is>
       </c>
-      <c r="H20" s="77" t="inlineStr">
+      <c r="H20" s="97" t="inlineStr">
         <is>
           <t>기능검사기(UK4S)</t>
         </is>
@@ -5311,7 +5311,7 @@
       <c r="O20" s="79" t="n">
         <v>3205000</v>
       </c>
-      <c r="P20" s="80" t="n">
+      <c r="P20" s="96" t="n">
         <v>3205000</v>
       </c>
       <c r="Q20" s="81" t="inlineStr">
@@ -5370,12 +5370,12 @@
         </is>
       </c>
       <c r="F21" s="67" t="n"/>
-      <c r="G21" s="68" t="inlineStr">
+      <c r="G21" s="98" t="inlineStr">
         <is>
           <t>SM-L715 MIC KEY</t>
         </is>
       </c>
-      <c r="H21" s="68" t="inlineStr">
+      <c r="H21" s="98" t="inlineStr">
         <is>
           <t>기능검사기(UK3S)</t>
         </is>
@@ -5407,7 +5407,7 @@
       <c r="O21" s="70" t="n">
         <v>3705000</v>
       </c>
-      <c r="P21" s="71" t="n">
+      <c r="P21" s="95" t="n">
         <v>3705000</v>
       </c>
       <c r="Q21" s="72" t="inlineStr">
@@ -5471,7 +5471,7 @@
           <t>SM-L715 MIC KEY</t>
         </is>
       </c>
-      <c r="H22" s="77" t="inlineStr">
+      <c r="H22" s="97" t="inlineStr">
         <is>
           <t>기능검사기(UK4S)</t>
         </is>
@@ -5503,7 +5503,7 @@
       <c r="O22" s="79" t="n">
         <v>3205000</v>
       </c>
-      <c r="P22" s="80" t="n">
+      <c r="P22" s="96" t="n">
         <v>3205000</v>
       </c>
       <c r="Q22" s="81" t="inlineStr">
@@ -5567,7 +5567,7 @@
           <t>SM-L715 MIC KEY</t>
         </is>
       </c>
-      <c r="H23" s="68" t="inlineStr">
+      <c r="H23" s="97" t="inlineStr">
         <is>
           <t>기능검사기(UK4S)</t>
         </is>
@@ -5599,7 +5599,7 @@
       <c r="O23" s="70" t="n">
         <v>3105000</v>
       </c>
-      <c r="P23" s="71" t="n">
+      <c r="P23" s="95" t="n">
         <v>3105000</v>
       </c>
       <c r="Q23" s="72" t="inlineStr">
@@ -5695,7 +5695,7 @@
       <c r="O24" s="79" t="n">
         <v>8900000</v>
       </c>
-      <c r="P24" s="80" t="n">
+      <c r="P24" s="96" t="n">
         <v>8900000</v>
       </c>
       <c r="Q24" s="81" t="inlineStr">
@@ -5791,7 +5791,7 @@
       <c r="O25" s="70" t="n">
         <v>5780000</v>
       </c>
-      <c r="P25" s="71" t="n">
+      <c r="P25" s="95" t="n">
         <v>5780000</v>
       </c>
       <c r="Q25" s="72" t="inlineStr">
@@ -5887,7 +5887,7 @@
       <c r="O26" s="79" t="n">
         <v>9230000</v>
       </c>
-      <c r="P26" s="80" t="n">
+      <c r="P26" s="96" t="n">
         <v>9230000</v>
       </c>
       <c r="Q26" s="81" t="inlineStr">
@@ -5983,7 +5983,7 @@
       <c r="O27" s="70" t="n">
         <v>5210000</v>
       </c>
-      <c r="P27" s="71" t="n">
+      <c r="P27" s="95" t="n">
         <v>5210000</v>
       </c>
       <c r="Q27" s="72" t="inlineStr">
@@ -6083,7 +6083,7 @@
       <c r="O28" s="79" t="n">
         <v>7640000</v>
       </c>
-      <c r="P28" s="80" t="n">
+      <c r="P28" s="96" t="n">
         <v>7640000</v>
       </c>
       <c r="Q28" s="81" t="inlineStr">
@@ -6179,7 +6179,7 @@
       <c r="O29" s="70" t="n">
         <v>8550000</v>
       </c>
-      <c r="P29" s="71" t="n">
+      <c r="P29" s="95" t="n">
         <v>8550000</v>
       </c>
       <c r="Q29" s="72" t="inlineStr">
@@ -6275,7 +6275,7 @@
       <c r="O30" s="79" t="n">
         <v>7550000</v>
       </c>
-      <c r="P30" s="80" t="n">
+      <c r="P30" s="96" t="n">
         <v>7550000</v>
       </c>
       <c r="Q30" s="81" t="inlineStr">
@@ -6371,7 +6371,7 @@
       <c r="O31" s="70" t="n">
         <v>7860000</v>
       </c>
-      <c r="P31" s="71" t="n">
+      <c r="P31" s="95" t="n">
         <v>7860000</v>
       </c>
       <c r="Q31" s="72" t="inlineStr">
@@ -6467,7 +6467,7 @@
       <c r="O32" s="79" t="n">
         <v>6850000</v>
       </c>
-      <c r="P32" s="80" t="n">
+      <c r="P32" s="96" t="n">
         <v>6850000</v>
       </c>
       <c r="Q32" s="81" t="inlineStr">
@@ -6563,7 +6563,7 @@
       <c r="O33" s="70" t="n">
         <v>7550000</v>
       </c>
-      <c r="P33" s="71" t="n">
+      <c r="P33" s="95" t="n">
         <v>7550000</v>
       </c>
       <c r="Q33" s="72" t="inlineStr">
@@ -6659,7 +6659,7 @@
       <c r="O34" s="79" t="n">
         <v>7270000</v>
       </c>
-      <c r="P34" s="80" t="n">
+      <c r="P34" s="96" t="n">
         <v>7270000</v>
       </c>
       <c r="Q34" s="81" t="inlineStr">
@@ -6755,7 +6755,7 @@
       <c r="O35" s="70" t="n">
         <v>1770000</v>
       </c>
-      <c r="P35" s="71" t="n">
+      <c r="P35" s="95" t="n">
         <v>5310000</v>
       </c>
       <c r="Q35" s="72" t="inlineStr">
@@ -6851,7 +6851,7 @@
       <c r="O36" s="79" t="n">
         <v>400000</v>
       </c>
-      <c r="P36" s="80" t="n">
+      <c r="P36" s="96" t="n">
         <v>400000</v>
       </c>
       <c r="Q36" s="81" t="inlineStr">
@@ -6947,7 +6947,7 @@
       <c r="O37" s="70" t="n">
         <v>3800000</v>
       </c>
-      <c r="P37" s="71" t="n">
+      <c r="P37" s="95" t="n">
         <v>3800000</v>
       </c>
       <c r="Q37" s="72" t="inlineStr">
@@ -7006,12 +7006,12 @@
         </is>
       </c>
       <c r="F38" s="76" t="n"/>
-      <c r="G38" s="77" t="inlineStr">
+      <c r="G38" s="98" t="inlineStr">
         <is>
           <t>SM-F971U MAIN LOWER HPCB</t>
         </is>
       </c>
-      <c r="H38" s="77" t="inlineStr">
+      <c r="H38" s="98" t="inlineStr">
         <is>
           <t>기능검사기 (UK4S)</t>
         </is>
@@ -7043,7 +7043,7 @@
       <c r="O38" s="79" t="n">
         <v>5020000</v>
       </c>
-      <c r="P38" s="80" t="n">
+      <c r="P38" s="96" t="n">
         <v>5020000</v>
       </c>
       <c r="Q38" s="81" t="inlineStr">
@@ -7139,7 +7139,7 @@
       <c r="O39" s="70" t="n">
         <v>247000</v>
       </c>
-      <c r="P39" s="71" t="n">
+      <c r="P39" s="95" t="n">
         <v>247000</v>
       </c>
       <c r="Q39" s="72" t="inlineStr">
@@ -7198,12 +7198,12 @@
         </is>
       </c>
       <c r="F40" s="76" t="n"/>
-      <c r="G40" s="77" t="inlineStr">
+      <c r="G40" s="98" t="inlineStr">
         <is>
           <t>SM-L716 BAROMETER</t>
         </is>
       </c>
-      <c r="H40" s="77" t="inlineStr">
+      <c r="H40" s="98" t="inlineStr">
         <is>
           <t>10기압 기능검사기(UK3S)</t>
         </is>
@@ -7235,7 +7235,7 @@
       <c r="O40" s="79" t="n">
         <v>6020000</v>
       </c>
-      <c r="P40" s="80" t="n">
+      <c r="P40" s="96" t="n">
         <v>6020000</v>
       </c>
       <c r="Q40" s="81" t="inlineStr">
@@ -7298,12 +7298,12 @@
           <t>PBA</t>
         </is>
       </c>
-      <c r="G41" s="68" t="inlineStr">
+      <c r="G41" s="98" t="inlineStr">
         <is>
           <t>SM-A27B USB PBA</t>
         </is>
       </c>
-      <c r="H41" s="68" t="inlineStr">
+      <c r="H41" s="98" t="inlineStr">
         <is>
           <t>성능검사기_케이스 제외</t>
         </is>
@@ -7335,7 +7335,7 @@
       <c r="O41" s="70" t="n">
         <v>3486800</v>
       </c>
-      <c r="P41" s="71" t="n">
+      <c r="P41" s="95" t="n">
         <v>6973600</v>
       </c>
       <c r="Q41" s="72" t="inlineStr">
@@ -7398,12 +7398,12 @@
           <t>PBA</t>
         </is>
       </c>
-      <c r="G42" s="77" t="inlineStr">
+      <c r="G42" s="98" t="inlineStr">
         <is>
           <t>SM-A27B USB PBA</t>
         </is>
       </c>
-      <c r="H42" s="77" t="inlineStr">
+      <c r="H42" s="98" t="inlineStr">
         <is>
           <t>VSWR검사기_케이스 제외</t>
         </is>
@@ -7435,7 +7435,7 @@
       <c r="O42" s="79" t="n">
         <v>2171200</v>
       </c>
-      <c r="P42" s="80" t="n">
+      <c r="P42" s="96" t="n">
         <v>4342400</v>
       </c>
       <c r="Q42" s="81" t="inlineStr">
@@ -7535,7 +7535,7 @@
       <c r="O43" s="70" t="n">
         <v>3486800</v>
       </c>
-      <c r="P43" s="71" t="n">
+      <c r="P43" s="95" t="n">
         <v>34868000</v>
       </c>
       <c r="Q43" s="72" t="inlineStr">
@@ -7635,7 +7635,7 @@
       <c r="O44" s="79" t="n">
         <v>2171200</v>
       </c>
-      <c r="P44" s="80" t="n">
+      <c r="P44" s="96" t="n">
         <v>13027200</v>
       </c>
       <c r="Q44" s="81" t="inlineStr">
@@ -7698,7 +7698,7 @@
           <t>PBA</t>
         </is>
       </c>
-      <c r="G45" s="68" t="inlineStr">
+      <c r="G45" s="97" t="inlineStr">
         <is>
           <t>SM-A27BE USB PBA</t>
         </is>
@@ -7735,7 +7735,7 @@
       <c r="O45" s="70" t="n">
         <v>3486800</v>
       </c>
-      <c r="P45" s="71" t="n">
+      <c r="P45" s="95" t="n">
         <v>38354800</v>
       </c>
       <c r="Q45" s="72" t="inlineStr">
@@ -7798,7 +7798,7 @@
           <t>PBA</t>
         </is>
       </c>
-      <c r="G46" s="77" t="inlineStr">
+      <c r="G46" s="97" t="inlineStr">
         <is>
           <t>SM-A27BE USB PBA</t>
         </is>
@@ -7835,7 +7835,7 @@
       <c r="O46" s="79" t="n">
         <v>2171200</v>
       </c>
-      <c r="P46" s="80" t="n">
+      <c r="P46" s="96" t="n">
         <v>15198400</v>
       </c>
       <c r="Q46" s="81" t="inlineStr">
@@ -7894,12 +7894,12 @@
         </is>
       </c>
       <c r="F47" s="67" t="n"/>
-      <c r="G47" s="68" t="inlineStr">
+      <c r="G47" s="98" t="inlineStr">
         <is>
           <t>VMF0971-0125003</t>
         </is>
       </c>
-      <c r="H47" s="68" t="inlineStr">
+      <c r="H47" s="98" t="inlineStr">
         <is>
           <t>VSWR 검사기- CASE 재활용</t>
         </is>
@@ -7931,7 +7931,7 @@
       <c r="O47" s="70" t="n">
         <v>2210000</v>
       </c>
-      <c r="P47" s="71" t="n">
+      <c r="P47" s="95" t="n">
         <v>2210000</v>
       </c>
       <c r="Q47" s="72" t="inlineStr">
@@ -8031,7 +8031,7 @@
       <c r="O48" s="79" t="n">
         <v>2080000</v>
       </c>
-      <c r="P48" s="80" t="n">
+      <c r="P48" s="96" t="n">
         <v>2080000</v>
       </c>
       <c r="Q48" s="81" t="inlineStr">
@@ -8131,7 +8131,7 @@
       <c r="O49" s="70" t="n">
         <v>2490000</v>
       </c>
-      <c r="P49" s="71" t="n">
+      <c r="P49" s="95" t="n">
         <v>2490000</v>
       </c>
       <c r="Q49" s="72" t="inlineStr">
@@ -8231,7 +8231,7 @@
       <c r="O50" s="79" t="n">
         <v>2140000</v>
       </c>
-      <c r="P50" s="80" t="n">
+      <c r="P50" s="96" t="n">
         <v>2140000</v>
       </c>
       <c r="Q50" s="81" t="inlineStr">
@@ -8331,7 +8331,7 @@
       <c r="O51" s="70" t="n">
         <v>2490000</v>
       </c>
-      <c r="P51" s="71" t="n">
+      <c r="P51" s="95" t="n">
         <v>2490000</v>
       </c>
       <c r="Q51" s="72" t="inlineStr">
@@ -8427,7 +8427,7 @@
       <c r="O52" s="79" t="n">
         <v>3420000</v>
       </c>
-      <c r="P52" s="80" t="n">
+      <c r="P52" s="96" t="n">
         <v>3420000</v>
       </c>
       <c r="Q52" s="81" t="inlineStr">
@@ -8523,7 +8523,7 @@
       <c r="O53" s="70" t="n">
         <v>5790000</v>
       </c>
-      <c r="P53" s="71" t="n">
+      <c r="P53" s="95" t="n">
         <v>5790000</v>
       </c>
       <c r="Q53" s="72" t="inlineStr">
@@ -8619,7 +8619,7 @@
       <c r="O54" s="79" t="n">
         <v>5690000</v>
       </c>
-      <c r="P54" s="80" t="n">
+      <c r="P54" s="96" t="n">
         <v>5690000</v>
       </c>
       <c r="Q54" s="81" t="inlineStr">
@@ -8715,7 +8715,7 @@
       <c r="O55" s="70" t="n">
         <v>5590000</v>
       </c>
-      <c r="P55" s="71" t="n">
+      <c r="P55" s="95" t="n">
         <v>5590000</v>
       </c>
       <c r="Q55" s="72" t="inlineStr">
@@ -8815,7 +8815,7 @@
       <c r="O56" s="79" t="n">
         <v>3400000</v>
       </c>
-      <c r="P56" s="80" t="n">
+      <c r="P56" s="96" t="n">
         <v>3400000</v>
       </c>
       <c r="Q56" s="81" t="inlineStr">
@@ -8911,7 +8911,7 @@
       <c r="O57" s="70" t="n">
         <v>3714000</v>
       </c>
-      <c r="P57" s="71" t="n">
+      <c r="P57" s="95" t="n">
         <v>3714000</v>
       </c>
       <c r="Q57" s="72" t="inlineStr">
@@ -9007,7 +9007,7 @@
       <c r="O58" s="79" t="n">
         <v>3614000</v>
       </c>
-      <c r="P58" s="80" t="n">
+      <c r="P58" s="96" t="n">
         <v>3614000</v>
       </c>
       <c r="Q58" s="81" t="inlineStr">
@@ -9103,7 +9103,7 @@
       <c r="O59" s="70" t="n">
         <v>3514000</v>
       </c>
-      <c r="P59" s="71" t="n">
+      <c r="P59" s="95" t="n">
         <v>3514000</v>
       </c>
       <c r="Q59" s="72" t="inlineStr">
@@ -9199,7 +9199,7 @@
       <c r="O60" s="79" t="n">
         <v>5590000</v>
       </c>
-      <c r="P60" s="80" t="n">
+      <c r="P60" s="96" t="n">
         <v>5590000</v>
       </c>
       <c r="Q60" s="81" t="inlineStr">
@@ -9258,12 +9258,12 @@
         </is>
       </c>
       <c r="F61" s="67" t="n"/>
-      <c r="G61" s="68" t="inlineStr">
+      <c r="G61" s="98" t="inlineStr">
         <is>
           <t>SM-F976U MAIN FRC</t>
         </is>
       </c>
-      <c r="H61" s="68" t="inlineStr">
+      <c r="H61" s="98" t="inlineStr">
         <is>
           <t>OS검사기_케이스포함</t>
         </is>
@@ -9295,7 +9295,7 @@
       <c r="O61" s="70" t="n">
         <v>5955000</v>
       </c>
-      <c r="P61" s="71" t="n">
+      <c r="P61" s="95" t="n">
         <v>5955000</v>
       </c>
       <c r="Q61" s="72" t="inlineStr">
@@ -9359,7 +9359,7 @@
           <t>SM-F976U MAIN FRC</t>
         </is>
       </c>
-      <c r="H62" s="77" t="inlineStr">
+      <c r="H62" s="97" t="inlineStr">
         <is>
           <t>OS검사기_MODIFY</t>
         </is>
@@ -9454,12 +9454,12 @@
         </is>
       </c>
       <c r="F63" s="67" t="n"/>
-      <c r="G63" s="68" t="inlineStr">
+      <c r="G63" s="98" t="inlineStr">
         <is>
           <t>SM-F976U MAIN FRC</t>
         </is>
       </c>
-      <c r="H63" s="68" t="inlineStr">
+      <c r="H63" s="98" t="inlineStr">
         <is>
           <t>TDR+IL검사기_케이스포함</t>
         </is>
@@ -9491,7 +9491,7 @@
       <c r="O63" s="70" t="n">
         <v>8625000</v>
       </c>
-      <c r="P63" s="71" t="n">
+      <c r="P63" s="95" t="n">
         <v>8625000</v>
       </c>
       <c r="Q63" s="72" t="inlineStr">
@@ -9555,7 +9555,7 @@
           <t>SM-F976U MAIN FRC</t>
         </is>
       </c>
-      <c r="H64" s="77" t="inlineStr">
+      <c r="H64" s="97" t="inlineStr">
         <is>
           <t>TDR+IL검사기_MODIFY</t>
         </is>
@@ -9691,7 +9691,7 @@
       <c r="O65" s="70" t="n">
         <v>2650000</v>
       </c>
-      <c r="P65" s="71" t="n">
+      <c r="P65" s="95" t="n">
         <v>5300000</v>
       </c>
       <c r="Q65" s="72" t="inlineStr">
@@ -9791,7 +9791,7 @@
       <c r="O66" s="79" t="n">
         <v>3486800</v>
       </c>
-      <c r="P66" s="80" t="n">
+      <c r="P66" s="96" t="n">
         <v>20920800</v>
       </c>
       <c r="Q66" s="81" t="inlineStr">
@@ -9891,7 +9891,7 @@
       <c r="O67" s="70" t="n">
         <v>2171200</v>
       </c>
-      <c r="P67" s="71" t="n">
+      <c r="P67" s="95" t="n">
         <v>6513600</v>
       </c>
       <c r="Q67" s="72" t="inlineStr">
@@ -9954,7 +9954,7 @@
           <t>PBA</t>
         </is>
       </c>
-      <c r="G68" s="77" t="inlineStr">
+      <c r="G68" s="97" t="inlineStr">
         <is>
           <t>SM-A27BE USB PBA</t>
         </is>
@@ -9991,7 +9991,7 @@
       <c r="O68" s="79" t="n">
         <v>3486800</v>
       </c>
-      <c r="P68" s="80" t="n">
+      <c r="P68" s="96" t="n">
         <v>10460400</v>
       </c>
       <c r="Q68" s="81" t="inlineStr">
@@ -10054,7 +10054,7 @@
           <t>PBA</t>
         </is>
       </c>
-      <c r="G69" s="68" t="inlineStr">
+      <c r="G69" s="97" t="inlineStr">
         <is>
           <t>SM-A27BE USB PBA</t>
         </is>
@@ -10091,7 +10091,7 @@
       <c r="O69" s="70" t="n">
         <v>2171200</v>
       </c>
-      <c r="P69" s="71" t="n">
+      <c r="P69" s="95" t="n">
         <v>4342400</v>
       </c>
       <c r="Q69" s="72" t="inlineStr">
@@ -10187,7 +10187,7 @@
       <c r="O70" s="79" t="n">
         <v>4120000</v>
       </c>
-      <c r="P70" s="80" t="n">
+      <c r="P70" s="96" t="n">
         <v>12360000</v>
       </c>
       <c r="Q70" s="81" t="inlineStr">
@@ -10251,7 +10251,7 @@
           <t>SM-F971U MAIN LOWER HPCB</t>
         </is>
       </c>
-      <c r="H71" s="68" t="inlineStr">
+      <c r="H71" s="97" t="inlineStr">
         <is>
           <t>기능검사기(UK4S)</t>
         </is>
@@ -10283,7 +10283,7 @@
       <c r="O71" s="70" t="n">
         <v>5390000</v>
       </c>
-      <c r="P71" s="71" t="n">
+      <c r="P71" s="95" t="n">
         <v>64680000</v>
       </c>
       <c r="Q71" s="72" t="inlineStr">
@@ -10379,7 +10379,7 @@
       <c r="O72" s="79" t="n">
         <v>5270000</v>
       </c>
-      <c r="P72" s="80" t="n">
+      <c r="P72" s="96" t="n">
         <v>52700000</v>
       </c>
       <c r="Q72" s="81" t="inlineStr">
@@ -10475,7 +10475,7 @@
       <c r="O73" s="70" t="n">
         <v>4220000</v>
       </c>
-      <c r="P73" s="71" t="n">
+      <c r="P73" s="95" t="n">
         <v>8440000</v>
       </c>
       <c r="Q73" s="72" t="inlineStr">
@@ -10539,7 +10539,7 @@
           <t>SM-F776U PROXIMITY</t>
         </is>
       </c>
-      <c r="H74" s="77" t="inlineStr">
+      <c r="H74" s="97" t="inlineStr">
         <is>
           <t>기능검사기(UK4)</t>
         </is>
@@ -10571,7 +10571,7 @@
       <c r="O74" s="79" t="n">
         <v>6250000</v>
       </c>
-      <c r="P74" s="80" t="n">
+      <c r="P74" s="96" t="n">
         <v>50000000</v>
       </c>
       <c r="Q74" s="81" t="inlineStr">
@@ -10667,7 +10667,7 @@
       <c r="O75" s="70" t="n">
         <v>21600000</v>
       </c>
-      <c r="P75" s="71" t="n">
+      <c r="P75" s="95" t="n">
         <v>21600000</v>
       </c>
       <c r="Q75" s="72" t="inlineStr">
@@ -10763,7 +10763,7 @@
       <c r="O76" s="79" t="n">
         <v>8625000</v>
       </c>
-      <c r="P76" s="80" t="n">
+      <c r="P76" s="96" t="n">
         <v>8625000</v>
       </c>
       <c r="Q76" s="81" t="inlineStr">
@@ -10859,7 +10859,7 @@
       <c r="O77" s="70" t="n">
         <v>5235000</v>
       </c>
-      <c r="P77" s="71" t="n">
+      <c r="P77" s="95" t="n">
         <v>5235000</v>
       </c>
       <c r="Q77" s="72" t="inlineStr">
@@ -10959,7 +10959,7 @@
       <c r="O78" s="79" t="n">
         <v>6335000</v>
       </c>
-      <c r="P78" s="80" t="n">
+      <c r="P78" s="96" t="n">
         <v>6335000</v>
       </c>
       <c r="Q78" s="81" t="inlineStr">
@@ -11055,7 +11055,7 @@
       <c r="O79" s="70" t="n">
         <v>4295000</v>
       </c>
-      <c r="P79" s="71" t="n">
+      <c r="P79" s="95" t="n">
         <v>4295000</v>
       </c>
       <c r="Q79" s="72" t="inlineStr">
@@ -11155,7 +11155,7 @@
       <c r="O80" s="79" t="n">
         <v>5235000</v>
       </c>
-      <c r="P80" s="80" t="n">
+      <c r="P80" s="96" t="n">
         <v>5235000</v>
       </c>
       <c r="Q80" s="81" t="inlineStr">
@@ -11255,7 +11255,7 @@
       <c r="O81" s="70" t="n">
         <v>6335000</v>
       </c>
-      <c r="P81" s="71" t="n">
+      <c r="P81" s="95" t="n">
         <v>6335000</v>
       </c>
       <c r="Q81" s="72" t="inlineStr">
@@ -11355,7 +11355,7 @@
       <c r="O82" s="79" t="n">
         <v>4295000</v>
       </c>
-      <c r="P82" s="80" t="n">
+      <c r="P82" s="96" t="n">
         <v>4295000</v>
       </c>
       <c r="Q82" s="81" t="inlineStr">
@@ -11451,7 +11451,7 @@
       <c r="O83" s="70" t="n">
         <v>4850000</v>
       </c>
-      <c r="P83" s="71" t="n">
+      <c r="P83" s="95" t="n">
         <v>4850000</v>
       </c>
       <c r="Q83" s="72" t="inlineStr">
@@ -11547,7 +11547,7 @@
       <c r="O84" s="79" t="n">
         <v>7761000</v>
       </c>
-      <c r="P84" s="80" t="n">
+      <c r="P84" s="96" t="n">
         <v>7761000</v>
       </c>
       <c r="Q84" s="81" t="inlineStr">
@@ -11643,7 +11643,7 @@
       <c r="O85" s="70" t="n">
         <v>400000</v>
       </c>
-      <c r="P85" s="71" t="n">
+      <c r="P85" s="95" t="n">
         <v>3200000</v>
       </c>
       <c r="Q85" s="72" t="inlineStr">
@@ -11739,7 +11739,7 @@
       <c r="O86" s="79" t="n">
         <v>5265000</v>
       </c>
-      <c r="P86" s="80" t="n">
+      <c r="P86" s="96" t="n">
         <v>5265000</v>
       </c>
       <c r="Q86" s="81" t="inlineStr">
@@ -11839,7 +11839,7 @@
       <c r="O87" s="70" t="n">
         <v>2490000</v>
       </c>
-      <c r="P87" s="71" t="n">
+      <c r="P87" s="95" t="n">
         <v>2490000</v>
       </c>
       <c r="Q87" s="72" t="inlineStr">
@@ -11935,7 +11935,7 @@
       <c r="O88" s="79" t="n">
         <v>2410000</v>
       </c>
-      <c r="P88" s="80" t="n">
+      <c r="P88" s="96" t="n">
         <v>2410000</v>
       </c>
       <c r="Q88" s="81" t="inlineStr">
@@ -12031,7 +12031,7 @@
       <c r="O89" s="70" t="n">
         <v>2210000</v>
       </c>
-      <c r="P89" s="71" t="n">
+      <c r="P89" s="95" t="n">
         <v>2210000</v>
       </c>
       <c r="Q89" s="72" t="inlineStr">
@@ -12127,7 +12127,7 @@
       <c r="O90" s="79" t="n">
         <v>7820000</v>
       </c>
-      <c r="P90" s="80" t="n">
+      <c r="P90" s="96" t="n">
         <v>15640000</v>
       </c>
       <c r="Q90" s="81" t="inlineStr">
@@ -12227,7 +12227,7 @@
       <c r="O91" s="70" t="n">
         <v>2880000</v>
       </c>
-      <c r="P91" s="71" t="n">
+      <c r="P91" s="95" t="n">
         <v>2880000</v>
       </c>
       <c r="Q91" s="72" t="inlineStr">
@@ -12323,7 +12323,7 @@
       <c r="O92" s="79" t="n">
         <v>2210000</v>
       </c>
-      <c r="P92" s="80" t="n">
+      <c r="P92" s="96" t="n">
         <v>2210000</v>
       </c>
       <c r="Q92" s="81" t="inlineStr">
@@ -12419,7 +12419,7 @@
       <c r="O93" s="70" t="n">
         <v>5850000</v>
       </c>
-      <c r="P93" s="71" t="n">
+      <c r="P93" s="95" t="n">
         <v>5850000</v>
       </c>
       <c r="Q93" s="72" t="inlineStr">
@@ -12519,7 +12519,7 @@
       <c r="O94" s="79" t="n">
         <v>2140000</v>
       </c>
-      <c r="P94" s="80" t="n">
+      <c r="P94" s="96" t="n">
         <v>8560000</v>
       </c>
       <c r="Q94" s="81" t="inlineStr">
@@ -12619,7 +12619,7 @@
       <c r="O95" s="70" t="n">
         <v>2040000</v>
       </c>
-      <c r="P95" s="71" t="n">
+      <c r="P95" s="95" t="n">
         <v>4080000</v>
       </c>
       <c r="Q95" s="72" t="inlineStr">
@@ -12719,7 +12719,7 @@
       <c r="O96" s="79" t="n">
         <v>2780000</v>
       </c>
-      <c r="P96" s="80" t="n">
+      <c r="P96" s="96" t="n">
         <v>8340000</v>
       </c>
       <c r="Q96" s="81" t="inlineStr">
@@ -12819,7 +12819,7 @@
       <c r="O97" s="70" t="n">
         <v>2680000</v>
       </c>
-      <c r="P97" s="71" t="n">
+      <c r="P97" s="95" t="n">
         <v>8040000</v>
       </c>
       <c r="Q97" s="72" t="inlineStr">
@@ -12915,7 +12915,7 @@
       <c r="O98" s="79" t="n">
         <v>3161</v>
       </c>
-      <c r="P98" s="80" t="n">
+      <c r="P98" s="96" t="n">
         <v>37932</v>
       </c>
       <c r="Q98" s="81" t="inlineStr">
@@ -12974,7 +12974,7 @@
         </is>
       </c>
       <c r="F99" s="67" t="n"/>
-      <c r="G99" s="68" t="inlineStr">
+      <c r="G99" s="97" t="inlineStr">
         <is>
           <t>SM-L715 BAROMETER</t>
         </is>
@@ -13011,7 +13011,7 @@
       <c r="O99" s="70" t="n">
         <v>4540</v>
       </c>
-      <c r="P99" s="71" t="n">
+      <c r="P99" s="95" t="n">
         <v>54480</v>
       </c>
       <c r="Q99" s="72" t="inlineStr">
@@ -13111,7 +13111,7 @@
       <c r="O100" s="79" t="n">
         <v>7000000</v>
       </c>
-      <c r="P100" s="80" t="n">
+      <c r="P100" s="96" t="n">
         <v>7000000</v>
       </c>
       <c r="Q100" s="81" t="inlineStr">
@@ -13207,7 +13207,7 @@
       <c r="O101" s="70" t="n">
         <v>8300000</v>
       </c>
-      <c r="P101" s="71" t="n">
+      <c r="P101" s="95" t="n">
         <v>8300000</v>
       </c>
       <c r="Q101" s="72" t="inlineStr">
@@ -13303,7 +13303,7 @@
       <c r="O102" s="79" t="n">
         <v>6440000</v>
       </c>
-      <c r="P102" s="80" t="n">
+      <c r="P102" s="96" t="n">
         <v>6440000</v>
       </c>
       <c r="Q102" s="81" t="inlineStr">
@@ -13399,7 +13399,7 @@
       <c r="O103" s="70" t="n">
         <v>6440000</v>
       </c>
-      <c r="P103" s="71" t="n">
+      <c r="P103" s="95" t="n">
         <v>6440000</v>
       </c>
       <c r="Q103" s="72" t="inlineStr">
@@ -13458,12 +13458,12 @@
         </is>
       </c>
       <c r="F104" s="76" t="n"/>
-      <c r="G104" s="77" t="inlineStr">
+      <c r="G104" s="97" t="inlineStr">
         <is>
           <t>ZNB-400</t>
         </is>
       </c>
-      <c r="H104" s="77" t="inlineStr">
+      <c r="H104" s="97" t="inlineStr">
         <is>
           <t>모듈검사기_케이스 제외</t>
         </is>
@@ -13495,7 +13495,7 @@
       <c r="O104" s="79" t="n">
         <v>4807000</v>
       </c>
-      <c r="P104" s="80" t="n">
+      <c r="P104" s="96" t="n">
         <v>4807000</v>
       </c>
       <c r="Q104" s="81" t="inlineStr">
@@ -13591,7 +13591,7 @@
       <c r="O105" s="70" t="n">
         <v>3648000</v>
       </c>
-      <c r="P105" s="71" t="n">
+      <c r="P105" s="95" t="n">
         <v>3648000</v>
       </c>
       <c r="Q105" s="72" t="inlineStr">
@@ -13685,7 +13685,7 @@
       <c r="O106" s="79" t="n">
         <v>3548000</v>
       </c>
-      <c r="P106" s="80" t="n">
+      <c r="P106" s="96" t="n">
         <v>3548000</v>
       </c>
       <c r="Q106" s="81" t="inlineStr">
@@ -13779,7 +13779,7 @@
       <c r="O107" s="70" t="n">
         <v>110000000</v>
       </c>
-      <c r="P107" s="71" t="n">
+      <c r="P107" s="95" t="n">
         <v>110000000</v>
       </c>
       <c r="Q107" s="72" t="inlineStr">
@@ -13873,7 +13873,7 @@
       <c r="O108" s="79" t="n">
         <v>23000000</v>
       </c>
-      <c r="P108" s="80" t="n">
+      <c r="P108" s="96" t="n">
         <v>23000000</v>
       </c>
       <c r="Q108" s="81" t="inlineStr">
@@ -13971,7 +13971,7 @@
       <c r="O109" s="70" t="n">
         <v>6000000</v>
       </c>
-      <c r="P109" s="71" t="n">
+      <c r="P109" s="95" t="n">
         <v>12000000</v>
       </c>
       <c r="Q109" s="72" t="inlineStr">
@@ -14055,7 +14055,7 @@
       <c r="O110" s="79" t="n">
         <v>6000000</v>
       </c>
-      <c r="P110" s="80" t="n">
+      <c r="P110" s="96" t="n">
         <v>12000000</v>
       </c>
       <c r="Q110" s="81" t="inlineStr">
@@ -15310,7 +15310,7 @@
           <t>업데이트: 2026-05-03 00:43</t>
         </is>
       </c>
-      <c r="AR2" s="108" t="inlineStr">
+      <c r="AR2" s="111" t="inlineStr">
         <is>
           <t>업데이트: 2026-05-02 01:43</t>
         </is>

</xml_diff>